<commit_message>
Demo web model with add more detail data
</commit_message>
<xml_diff>
--- a/service_model_training_data_template.xlsx
+++ b/service_model_training_data_template.xlsx
@@ -503,6 +503,16 @@
           <t>パスワードを忘れました</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>No worries! Tap 'Forgot Password' on the login screen, enter your email, and we'll send a reset link within 1 minute.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ご安心ください！ログイン画面の「パスワードを忘れた」をタップし、メールアドレスを入力してください。1分以内にリセットリンクをお送りします。</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="C5" t="inlineStr">
@@ -515,6 +525,16 @@
           <t>ログインできません</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Let's get you back in! First try resetting your password via Settings &gt; Account &gt; Reset Password. If that doesn't work, check if your account email is correct.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>アカウントに戻れるようお手伝いします！まず設定 &gt; アカウント &gt; パスワードリセットをお試しください。それでもダメな場合は、メールアドレスが正しいかご確認ください。</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="C6" t="inlineStr">
@@ -527,6 +547,16 @@
           <t>パスワードを変更したい</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Your password may have expired or been changed. Try the 'Forgot Password' option on the login screen to create a new one.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>パスワードの有効期限が切れているか、変更された可能性があります。ログイン画面の「パスワードを忘れた」から新しいパスワードを作成してください。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="C7" t="inlineStr">
@@ -539,6 +569,16 @@
           <t>アカウントにアクセスできない</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Account lockouts happen after too many failed attempts. Wait 15 minutes and try again, or reset your password via email to unlock immediately.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ログイン試行回数が多すぎるとアカウントがロックされます。15分待ってから再試行するか、メールでパスワードをリセットして即座にロック解除できます。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="C8" t="inlineStr">
@@ -551,6 +591,16 @@
           <t>パスワードがわからない</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>To recover your account: go to the login screen &gt; tap 'Forgot Password' &gt; enter your registered email. A recovery link will be sent within minutes.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>アカウントを復旧するには：ログイン画面 &gt; 「パスワードを忘れた」をタップ &gt; 登録メールアドレスを入力。数分以内に復旧リンクが届きます。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="C9" t="inlineStr">
@@ -558,6 +608,16 @@
           <t>password reset please</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Absolutely! Go to Settings &gt; Account &gt; Reset Password. We'll send a secure link to your email right away.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>もちろんです！設定 &gt; アカウント &gt; パスワードリセットへ進んでください。メールにリンクをすぐにお送りします。</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -602,6 +662,16 @@
           <t>解約したい</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>To unsubscribe: Settings &gt; Subscription &gt; Cancel Plan. Your access continues until the current billing cycle ends.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>解約するには：設定 &gt; サブスクリプション &gt; キャンセル。現在の請求期間が終わるまでアクセスは継続されます。</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="C12" t="inlineStr">
@@ -614,6 +684,16 @@
           <t>退会方法を教えてください</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>To cancel your plan: Settings &gt; Subscription &gt; Cancel Plan. No immediate cutoff — you'll keep access until your current period ends.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>プランのキャンセル：設定 &gt; サブスクリプション &gt; キャンセル。すぐに停止されることはなく、現在の期間終了までご利用いただけます。</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="C13" t="inlineStr">
@@ -626,6 +706,16 @@
           <t>課金を止めてください</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>To stop charges: go to Settings &gt; Subscription &gt; Cancel Plan. Future charges will stop, and you keep access until the period ends.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>課金を停止するには：設定 &gt; サブスクリプション &gt; キャンセル。今後の課金は停止され、期間終了までアクセスは継続されます。</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -670,6 +760,16 @@
           <t>領収書がほしい</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>You can download receipts from Settings &gt; Billing &gt; Invoice History. Each transaction has a downloadable PDF receipt.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>領収書は設定 &gt; 請求 &gt; 請求履歴からダウンロードできます。各取引にPDF領収書があります。</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="C16" t="inlineStr">
@@ -682,6 +782,16 @@
           <t>支払い方法を変更したい</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>To update payment method: Settings &gt; Billing &gt; Payment Methods &gt; Add/Edit. You can add credit cards, debit cards, or PayPal.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>支払い方法の更新：設定 &gt; 請求 &gt; 支払い方法 &gt; 追加/編集。クレジットカード、デビットカード、PayPalを追加できます。</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -726,6 +836,16 @@
           <t>保存したアイテムはどこ？</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Your saved items are at: Home &gt; Saved tab (bookmark icon). You can also search within saved items.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>保存したアイテムは：ホーム &gt; 保存タブ（ブックマークアイコン）にあります。保存アイテム内での検索も可能です。</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -770,6 +890,16 @@
           <t>バグを見つけました</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Thanks for reporting! Please describe the bug at Settings &gt; Help &gt; Report a Bug. Include screenshots if possible — it helps us fix it faster.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>ご報告ありがとうございます！設定 &gt; ヘルプ &gt; バグを報告 で詳細をお知らせください。スクリーンショットがあると早く修正できます。</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="C21" t="inlineStr">
@@ -782,6 +912,16 @@
           <t>アプリが動かない</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Sorry to hear that! Try these first: 1) Force close and reopen 2) Update the app 3) Restart your device. If it persists, report at Settings &gt; Help &gt; Report a Bug.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>申し訳ございません！まずお試しください：1) 強制終了して再起動 2) アプリを更新 3) デバイスを再起動。改善しない場合は設定 &gt; ヘルプ &gt; バグを報告からご連絡ください。</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="C22" t="inlineStr">
@@ -794,6 +934,16 @@
           <t>正常に動作しません</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Sorry about that! Can you tell us what's not working? In the meantime, try updating the app and restarting your device. Report details at Settings &gt; Help &gt; Report a Bug.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>ご不便をおかけして申し訳ございません！何が動作していないかお知らせください。アプリの更新とデバイスの再起動もお試しください。詳細は設定 &gt; ヘルプ &gt; バグを報告へ。</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -838,6 +988,16 @@
           <t>サポートに繋いでください</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>I'll connect you now! Please fill out our support form at Settings &gt; Help &gt; Contact Support. A team member will respond within 24 hours.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>すぐにおつなぎします！設定 &gt; ヘルプ &gt; サポートに連絡のフォームにご記入ください。24時間以内にチームメンバーが対応します。</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="C25" t="inlineStr">
@@ -850,6 +1010,16 @@
           <t>直接相談したい</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Absolutely! Our support team is ready to help. Please reach out at Settings &gt; Help &gt; Contact Support, or say what your issue is and I'll try my best first.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>もちろんです！サポートチームがお手伝いします。設定 &gt; ヘルプ &gt; サポートに連絡からご連絡ください。まず私でお手伝いできることがあればお知らせください。</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -894,6 +1064,16 @@
           <t>冗談を教えて</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Ha! I wish I could tell jokes, but I'm only trained for app support. I can help with accounts, billing, features, or bugs. What do you need?</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>冗談を言えたらいいのですが、アプリサポート専用です！アカウント、請求、機能、バグについてお手伝いできます。何かお困りですか？</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="C28" t="inlineStr">
@@ -906,6 +1086,16 @@
           <t>今何時？</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>I can't tell time, but I can help with your account! Try asking about passwords, subscriptions, billing, or app features.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>時間はわかりませんが、アカウントのお手伝いはできます！パスワード、サブスクリプション、請求、アプリ機能についてお聞きください。</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="C29" t="inlineStr">
@@ -918,6 +1108,16 @@
           <t>昨日の試合の結果は？</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>I don't follow sports, but I'm great at app support! Ask me about your account, billing, features, or report a bug.</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>スポーツには詳しくないですが、アプリサポートは得意です！アカウント、請求、機能、バグ報告についてお聞きください。</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="C30" t="inlineStr">
@@ -930,6 +1130,16 @@
           <t>ピザを注文して</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>I can't order pizza, but I can help with your app! Try asking about passwords, subscriptions, billing, or features.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>ピザの注文はできませんが、アプリのお手伝いならできます！パスワード、サブスクリプション、請求、機能についてお聞きください。</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -974,6 +1184,16 @@
           <t>やあ</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Hi there! Welcome to support. I can help with accounts, billing, subscriptions, app features, and bug reports. What's on your mind?</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>こんにちは！サポートへようこそ。アカウント、請求、サブスクリプション、機能、バグ報告についてお手伝いできます。何かお困りですか？</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="C33" t="inlineStr">
@@ -986,6 +1206,16 @@
           <t>おはようございます</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Hey! I'm your support assistant. Ask me about passwords, billing, subscriptions, features, or report a bug. How can I help?</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>やあ！サポートアシスタントです。パスワード、請求、サブスクリプション、機能、バグ報告についてお聞きください。</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="C34" t="inlineStr">
@@ -998,6 +1228,16 @@
           <t>こんばんは</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Hey there! Ready to help. I can assist with accounts, subscriptions, billing, features, and bug reports. What do you need?</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>やあ！お手伝いの準備ができています。アカウント、サブスクリプション、請求、機能、バグ報告について対応できます。</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="C35" t="inlineStr">
@@ -1010,6 +1250,16 @@
           <t>すみません</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Of course I can help! I'm your AI support assistant. Ask about passwords, billing, subscriptions, features, or bugs.</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>もちろんお手伝いできます！AIサポートアシスタントです。パスワード、請求、サブスクリプション、機能、バグについてお聞きください。</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="C36" t="inlineStr">
@@ -1022,6 +1272,16 @@
           <t>助けてください</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Hello! I'm here to help. You can ask me about accounts, billing, subscriptions, app features, or report issues.</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>こんにちは！お手伝いいたします。アカウント、請求、サブスクリプション、機能、問題報告についてお聞きください。</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="C37" t="inlineStr">
@@ -1034,6 +1294,16 @@
           <t>ちょっといいですか</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Good morning! Welcome to support. How can I assist you today? I handle accounts, billing, features, and bug reports.</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>おはようございます！サポートへようこそ。今日は何かお手伝いできますか？アカウント、請求、機能、バグ報告に対応しています。</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="C38" t="inlineStr">
@@ -1046,6 +1316,16 @@
           <t>よろしくお願いします</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Good afternoon! I'm your support bot. Ask about passwords, subscriptions, billing, or app features. What do you need?</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>こんにちは！サポートボットです。パスワード、サブスクリプション、請求、機能についてお聞きください。</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="C39" t="inlineStr">
@@ -1058,6 +1338,16 @@
           <t>お世話になります</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Good evening! I'm available 24/7 to help with accounts, billing, subscriptions, and features. What can I help with?</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>こんばんは！アカウント、請求、サブスクリプション、機能について24時間対応しています。何かお手伝いできますか？</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="C40" t="inlineStr">
@@ -1070,6 +1360,16 @@
           <t>手伝ってもらえますか</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Absolutely! I can help with account issues, billing, subscriptions, features, and bug reports. What do you need?</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>もちろんです！アカウント、請求、サブスクリプション、機能、バグ報告についてお手伝いできます。何かお困りですか？</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="C41" t="inlineStr">
@@ -1082,6 +1382,16 @@
           <t>質問があります</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>I'm here to assist! Ask me about passwords, billing, subscriptions, app features, or report a problem.</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>お手伝いいたします！パスワード、請求、サブスクリプション、機能、問題報告についてお聞きください。</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="C42" t="inlineStr">
@@ -1094,6 +1404,16 @@
           <t>誰かいますか</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Yes, I'm here! I'm your AI support assistant. How can I help you today?</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>はい、ここにいます！AIサポートアシスタントです。今日は何かお手伝いできますか？</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="C43" t="inlineStr">
@@ -1106,6 +1426,16 @@
           <t>お願いがあります</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>I'm happy to help! What do you need assistance with? I can handle accounts, billing, features, and bugs.</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>喜んでお手伝いします！何についてのご質問ですか？アカウント、請求、機能、バグに対応しています。</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="C44" t="inlineStr">
@@ -1118,6 +1448,16 @@
           <t>何ができますか</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>I can help with: accounts &amp; passwords, subscriptions, billing, app features, and bug reports. What would you like?</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>お手伝いできること：アカウント・パスワード、サブスクリプション、請求、機能、バグ報告。何をお知りになりたいですか？</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="C45" t="inlineStr">
@@ -1130,6 +1470,16 @@
           <t>聞きたいことがあります</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Great, I'm ready for your question! I handle accounts, billing, subscriptions, features, and technical issues.</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>ご質問をどうぞ！アカウント、請求、サブスクリプション、機能、技術的な問題に対応しています。</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="C46" t="inlineStr">
@@ -1142,6 +1492,16 @@
           <t>ボットさん</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Hi! I'm your support bot. Ask me anything about the app — accounts, billing, features, subscriptions, or bugs!</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>こんにちは！サポートボットです。アプリについて何でもお聞きください。アカウント、請求、機能、サブスクリプション、バグなど！</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="C47" t="inlineStr">
@@ -1154,6 +1514,16 @@
           <t>ヘルプ</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>I'm here to help! What do you need? I can assist with accounts, passwords, billing, subscriptions, features, and bugs.</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>お手伝いします！何が必要ですか？アカウント、パスワード、請求、サブスクリプション、機能、バグに対応しています。</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="C48" t="inlineStr">
@@ -1166,6 +1536,16 @@
           <t>始めましょう</t>
         </is>
       </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Let's get started! Tell me what you need help with. I can handle accounts, billing, subscriptions, features, and bugs.</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>始めましょう！何についてお手伝いが必要ですか？アカウント、請求、サブスクリプション、機能、バグに対応しています。</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="C49" t="inlineStr">
@@ -1178,6 +1558,16 @@
           <t>いますか</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Yes, I'm here! What can I help you with today? Ask about accounts, billing, features, or report a problem.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>はい、ここにいます！今日は何かお手伝いできますか？アカウント、請求、機能、問題報告についてお聞きください。</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="C50" t="inlineStr">
@@ -1190,6 +1580,16 @@
           <t>サポートお願いします</t>
         </is>
       </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Of course! I'm your support assistant. Ask me about passwords, billing, subscriptions, features, or report issues.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>もちろんです！サポートアシスタントです。パスワード、請求、サブスクリプション、機能、問題報告についてお聞きください。</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1212,6 +1612,16 @@
           <t>パスワードが思い出せない</t>
         </is>
       </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>That happens! Just tap 'Forgot Password' on the login screen. We'll email you a secure link to create a new password.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>よくあることです！ログイン画面の「パスワードを忘れた」をタップしてください。新しいパスワードを作成するためのリンクをメールでお送りします。</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1234,6 +1644,16 @@
           <t>ログインパスワードの変更方法は？</t>
         </is>
       </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>To change your login password: Settings &gt; Account &gt; Change Password. You'll need to verify your current password first.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>ログインパスワードの変更方法：設定 &gt; アカウント &gt; パスワード変更。まず現在のパスワードの確認が必要です。</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1256,6 +1676,16 @@
           <t>パスワードリセットがうまくいかない</t>
         </is>
       </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>If the reset isn't working: 1) Check spam folder 2) Make sure the link hasn't expired (30 min) 3) Request a new link. Still stuck? Say 'I need human help'.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>リセットがうまくいかない場合：1) 迷惑メールを確認 2) リンクの有効期限（30分）を確認 3) 新しいリンクをリクエスト。解決しない場合は「人と話したい」とお伝えください。</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1278,6 +1708,16 @@
           <t>パスワードを更新したい</t>
         </is>
       </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>To update your password: Settings &gt; Account &gt; Change Password. Use at least 8 characters with numbers and symbols for best security.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>パスワードを更新するには：設定 &gt; アカウント &gt; パスワード変更。セキュリティのため、8文字以上で数字と記号を含めてください。</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1300,6 +1740,16 @@
           <t>パスワードはどこで変更できますか？</t>
         </is>
       </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>You can change your password at: Settings &gt; Account &gt; Change Password. Or use 'Forgot Password' on the login screen.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>パスワードの変更は：設定 &gt; アカウント &gt; パスワード変更。またはログイン画面の「パスワードを忘れた」をご利用ください。</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1322,6 +1772,16 @@
           <t>パスワードの有効期限が切れました</t>
         </is>
       </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Your password has expired for security. Reset it via Settings &gt; Account &gt; Reset Password, or tap 'Forgot Password' at login.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>セキュリティのためパスワードが期限切れです。設定 &gt; アカウント &gt; パスワードリセット、またはログイン時の「パスワードを忘れた」からリセットしてください。</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1344,6 +1804,16 @@
           <t>パスワードを間違えてロックされた</t>
         </is>
       </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Account locks happen after multiple failed attempts. Wait 15 minutes and try again, or reset your password via email to unlock immediately.</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>複数回のログイン失敗でアカウントがロックされます。15分待って再試行するか、メールでパスワードをリセットして即座に解除できます。</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1366,6 +1836,16 @@
           <t>パスワードエラーが出続けます</t>
         </is>
       </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Password errors usually mean it's incorrect or expired. Try 'Forgot Password' on the login screen to create a new one.</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>パスワードエラーは通常、パスワードが間違っているか期限切れです。ログイン画面の「パスワードを忘れた」から新しいパスワードを作成してください。</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1388,6 +1868,16 @@
           <t>アカウントに戻れるようにして</t>
         </is>
       </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Let's get you back in! Go to the login screen &gt; tap 'Forgot Password' &gt; enter your email. A recovery link will arrive within minutes.</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>アカウントに戻れるようお手伝いします！ログイン画面 &gt; 「パスワードを忘れた」&gt; メールアドレスを入力。数分以内に復旧リンクが届きます。</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1410,6 +1900,16 @@
           <t>ログイン情報を変更したい</t>
         </is>
       </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>To change your login info: Settings &gt; Account &gt; Change Password. You'll need your current password for verification.</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>ログイン情報の変更：設定 &gt; アカウント &gt; パスワード変更。確認のため現在のパスワードが必要です。</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1432,6 +1932,16 @@
           <t>認証情報を忘れました</t>
         </is>
       </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>No problem! Tap 'Forgot Password' on the login screen and enter your registered email. We'll send a reset link right away.</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>大丈夫です！ログイン画面の「パスワードを忘れた」をタップし、登録メールアドレスを入力してください。リセットリンクをすぐにお送りします。</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1454,6 +1964,16 @@
           <t>新しいパスワードを設定するには</t>
         </is>
       </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>To set a new password: Settings &gt; Account &gt; Change Password. Choose at least 8 characters with mixed case, numbers, and symbols.</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>新しいパスワードの設定：設定 &gt; アカウント &gt; パスワード変更。8文字以上で大小文字・数字・記号を含めてください。</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1476,6 +1996,16 @@
           <t>サービスの支払いを止めたい</t>
         </is>
       </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>To stop paying: Settings &gt; Subscription &gt; Cancel Plan. You won't be charged again after your current billing period ends.</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>支払いを停止するには：設定 &gt; サブスクリプション &gt; キャンセル。現在の請求期間終了後は課金されません。</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1498,6 +2028,16 @@
           <t>会員を解約するには？</t>
         </is>
       </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>To end your membership: Settings &gt; Subscription &gt; Cancel Plan. Your access continues until the billing period ends.</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>メンバーシップを終了するには：設定 &gt; サブスクリプション &gt; キャンセル。請求期間終了までアクセスは継続されます。</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1520,6 +2060,16 @@
           <t>アカウントのサブスクをキャンセルしたい</t>
         </is>
       </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>To cancel: Settings &gt; Subscription &gt; Cancel Plan. Follow the confirmation steps and you're all set.</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>キャンセルするには：設定 &gt; サブスクリプション &gt; キャンセル。確認手順に従えば完了です。</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1542,6 +2092,16 @@
           <t>更新したくありません</t>
         </is>
       </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>To stop renewal: Settings &gt; Subscription &gt; Cancel Plan. Your plan won't auto-renew and you keep access until the current period ends.</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>自動更新を停止するには：設定 &gt; サブスクリプション &gt; キャンセル。自動更新が停止され、現在の期間終了まで利用できます。</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1564,6 +2124,16 @@
           <t>月額課金を止めてください</t>
         </is>
       </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>To stop monthly payments: Settings &gt; Subscription &gt; Cancel Plan. No more charges after the current cycle ends.</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>月額支払いを停止するには：設定 &gt; サブスクリプション &gt; キャンセル。現在の期間終了後は課金されません。</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1586,6 +2156,16 @@
           <t>プランのキャンセルはどこで？</t>
         </is>
       </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>You can cancel at: Settings &gt; Subscription &gt; Cancel Plan. The process takes less than a minute.</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>キャンセルは：設定 &gt; サブスクリプション &gt; キャンセル から行えます。1分もかかりません。</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1608,6 +2188,16 @@
           <t>無料プランに戻したい</t>
         </is>
       </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>To downgrade to free: Settings &gt; Subscription &gt; Change Plan &gt; Free. You'll keep your data and basic features.</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>無料プランへダウングレード：設定 &gt; サブスクリプション &gt; プラン変更 &gt; 無料。データと基本機能はそのまま保持されます。</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1630,6 +2220,16 @@
           <t>プレミアムの登録を終了したい</t>
         </is>
       </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>To end premium: Settings &gt; Subscription &gt; Cancel Plan. You'll switch to the free plan after your current period ends.</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>プレミアムを終了するには：設定 &gt; サブスクリプション &gt; キャンセル。現在の期間終了後に無料プランに切り替わります。</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1652,6 +2252,16 @@
           <t>サブスクリプションを解除したい</t>
         </is>
       </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>To remove your subscription: Settings &gt; Subscription &gt; Cancel Plan. Confirmation email will be sent to you.</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>サブスクリプションを解除するには：設定 &gt; サブスクリプション &gt; キャンセル。確認メールが送信されます。</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1674,6 +2284,16 @@
           <t>このサービスはもう不要です</t>
         </is>
       </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>To cancel since you no longer need the service: Settings &gt; Subscription &gt; Cancel Plan. We're sorry to see you go!</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>サービスが不要になった場合のキャンセル：設定 &gt; サブスクリプション &gt; キャンセル。ご利用ありがとうございました！</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1696,6 +2316,16 @@
           <t>すべての登録を解除して</t>
         </is>
       </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>To unsubscribe from everything: Settings &gt; Subscription &gt; Cancel Plan. For email notifications, also check Settings &gt; Notifications.</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>すべての解約：設定 &gt; サブスクリプション &gt; キャンセル。メール通知については設定 &gt; 通知もご確認ください。</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1718,6 +2348,16 @@
           <t>更新をキャンセルしてください</t>
         </is>
       </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>To cancel renewal: Settings &gt; Subscription &gt; Cancel Plan. Your plan won't renew and access continues until the end of the current period.</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>更新をキャンセルするには：設定 &gt; サブスクリプション &gt; キャンセル。更新されず、現在の期間終了までアクセスは継続されます。</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1740,6 +2380,16 @@
           <t>予期しない請求があります</t>
         </is>
       </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Unexpected charges may be from a plan upgrade or trial ending. Check Settings &gt; Billing for details. If it's an error, we can process a refund within 14 days.</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>予期しない請求はプランのアップグレードやトライアル終了の可能性があります。設定 &gt; 請求で詳細を確認してください。誤りの場合は14日以内に返金処理が可能です。</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1762,6 +2412,16 @@
           <t>請求書はどこで確認できますか？</t>
         </is>
       </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>View your invoices at: Settings &gt; Billing &gt; Invoice History. You can download PDFs for each billing period.</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>請求書の確認：設定 &gt; 請求 &gt; 請求履歴。各請求期間のPDFをダウンロードできます。</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1784,6 +2444,16 @@
           <t>過剰請求されました</t>
         </is>
       </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Sorry about the overcharge! Check Settings &gt; Billing for payment details. If it's incorrect, we can issue a refund within 14 days. Say 'I need human help' for urgent cases.</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>過大請求について申し訳ございません！設定 &gt; 請求で支払い詳細をご確認ください。誤りの場合は14日以内に返金いたします。緊急の場合は「人と話したい」とお伝えください。</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1806,6 +2476,16 @@
           <t>次の請求日はいつですか？</t>
         </is>
       </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Your next billing date is shown at Settings &gt; Billing &gt; Subscription Details. You'll also receive an email reminder 3 days before.</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>次回の請求日は設定 &gt; 請求 &gt; サブスクリプション詳細に表示されています。請求日の3日前にメールでもお知らせします。</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1828,6 +2508,16 @@
           <t>返金してもらえますか？</t>
         </is>
       </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Refunds can be processed within 14 days of purchase. Go to Settings &gt; Billing &gt; select the transaction &gt; Request Refund. Or say 'I need human help' for assistance.</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>購入から14日以内であれば返金可能です。設定 &gt; 請求 &gt; 該当取引を選択 &gt; 返金リクエスト。サポートが必要な場合は「人と話したい」とお伝えください。</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1850,6 +2540,16 @@
           <t>年間払いに変更するには？</t>
         </is>
       </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>To switch to annual billing: Settings &gt; Billing &gt; Change Plan &gt; Annual. You'll save up to 20% compared to monthly!</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>年額課金への切り替え：設定 &gt; 請求 &gt; プラン変更 &gt; 年額。月額と比べて最大20%お得です！</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1872,6 +2572,16 @@
           <t>クレジットカードが拒否されました</t>
         </is>
       </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>If your card was declined: 1) Verify card details are correct 2) Check with your bank 3) Try a different payment method at Settings &gt; Billing &gt; Payment Methods.</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>カードが拒否された場合：1) カード情報が正しいか確認 2) 銀行にお問い合わせ 3) 設定 &gt; 請求 &gt; 支払い方法で別の方法をお試しください。</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1894,6 +2604,16 @@
           <t>プレミアムプランはいくらですか？</t>
         </is>
       </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Premium plan pricing is shown at Settings &gt; Subscription &gt; View Plans. We offer monthly and annual options with different features.</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>プレミアムプランの価格は設定 &gt; サブスクリプション &gt; プラン一覧でご確認いただけます。月額と年額のオプションがあります。</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1916,6 +2636,16 @@
           <t>請求先住所を変更したい</t>
         </is>
       </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>To change billing address: Settings &gt; Billing &gt; Billing Address &gt; Edit. Update your address and save.</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>請求先住所の変更：設定 &gt; 請求 &gt; 請求先住所 &gt; 編集。住所を更新して保存してください。</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1938,6 +2668,16 @@
           <t>支払い失敗なのにお金が引かれた</t>
         </is>
       </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>If payment failed but money was taken, it usually resolves within 3-5 business days. If not, contact your bank or say 'I need human help' for immediate assistance.</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>支払い失敗でお金が引かれた場合、通常3〜5営業日以内に解決します。解決しない場合は銀行にお問い合わせいただくか、「人と話したい」とお伝えください。</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1960,6 +2700,16 @@
           <t>プロモーションコードの適用方法は？</t>
         </is>
       </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>To apply a promo code: Settings &gt; Billing &gt; Apply Promo Code. Enter the code and tap Apply. Discount will be applied to your next billing.</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>プロモコードの適用：設定 &gt; 請求 &gt; プロモコード適用。コードを入力して適用をタップ。割引は次回の請求に反映されます。</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1982,6 +2732,16 @@
           <t>明細付きの領収書が必要です</t>
         </is>
       </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Itemized receipts are available at Settings &gt; Billing &gt; Invoice History. Select any transaction and tap 'Download Detailed Receipt'.</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>明細付き領収書は設定 &gt; 請求 &gt; 請求履歴からご利用いただけます。取引を選択し「詳細領収書をダウンロード」をタップしてください。</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2004,6 +2764,16 @@
           <t>通知を有効にするには？</t>
         </is>
       </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>To enable notifications: Settings &gt; Notifications &gt; toggle on. You can customize which notifications you receive.</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>通知を有効にするには：設定 &gt; 通知 &gt; オンに切り替え。受け取る通知の種類をカスタマイズできます。</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2026,6 +2796,16 @@
           <t>設定はどこですか？</t>
         </is>
       </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Settings can be found by tapping the gear icon in the top-right corner of the home screen, or via the menu &gt; Settings.</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>設定はホーム画面右上の歯車アイコンをタップするか、メニュー &gt; 設定からアクセスできます。</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2048,6 +2828,16 @@
           <t>データをエクスポートするには？</t>
         </is>
       </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>To export your data: Settings &gt; Privacy &gt; Export Data. You'll receive a download link via email within 24 hours.</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>データのエクスポート：設定 &gt; プライバシー &gt; データエクスポート。24時間以内にメールでダウンロードリンクが届きます。</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2070,6 +2860,16 @@
           <t>オフラインモードは使えますか？</t>
         </is>
       </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Yes! To use offline mode: Settings &gt; General &gt; Offline Mode. Downloaded content will be available without internet.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>はい！オフラインモードの利用：設定 &gt; 一般 &gt; オフラインモード。ダウンロード済みコンテンツがインターネットなしで利用可能です。</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2092,6 +2892,16 @@
           <t>言語を変更するには？</t>
         </is>
       </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>To change language: Settings &gt; General &gt; Language. Select your preferred language and restart the app.</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>言語の変更：設定 &gt; 一般 &gt; 言語。希望する言語を選択してアプリを再起動してください。</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2114,6 +2924,16 @@
           <t>プロフィールを共有するには？</t>
         </is>
       </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>To share your profile: go to your Profile page &gt; tap the Share icon (top-right). You can copy the link or share directly.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>プロフィールの共有：プロフィールページ &gt; 共有アイコン（右上）をタップ。リンクをコピーするか直接共有できます。</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2136,6 +2956,16 @@
           <t>検索機能はありますか？</t>
         </is>
       </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Yes! Tap the search icon (magnifying glass) at the top of any screen. You can search content, settings, and help articles.</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>はい！画面上部の検索アイコン（虫眼鏡）をタップしてください。コンテンツ、設定、ヘルプ記事を検索できます。</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2158,6 +2988,16 @@
           <t>履歴を削除するには？</t>
         </is>
       </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>To delete history: Settings &gt; Privacy &gt; Clear History. You can choose to clear all or select specific items.</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>履歴の削除：設定 &gt; プライバシー &gt; 履歴を消去。すべて消去するか、特定の項目を選択できます。</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2180,6 +3020,16 @@
           <t>デバイス間で同期できますか？</t>
         </is>
       </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Yes! Sign in with the same account on multiple devices. Your data syncs automatically via Settings &gt; Account &gt; Sync.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>はい！複数のデバイスで同じアカウントにログインしてください。設定 &gt; アカウント &gt; 同期でデータが自動同期されます。</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2202,6 +3052,16 @@
           <t>二段階認証の設定方法は？</t>
         </is>
       </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>To set up 2FA: Settings &gt; Security &gt; Two-Factor Authentication &gt; Enable. You'll need an authenticator app like Google Authenticator.</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>二段階認証の設定：設定 &gt; セキュリティ &gt; 二段階認証 &gt; 有効化。Google Authenticatorなどの認証アプリが必要です。</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2224,6 +3084,16 @@
           <t>ダッシュボードをカスタマイズするには？</t>
         </is>
       </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>To customize your dashboard: Home &gt; tap Edit (pencil icon). Drag widgets to rearrange, and toggle visibility on/off.</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>ダッシュボードのカスタマイズ：ホーム &gt; 編集（鉛筆アイコン）をタップ。ウィジェットをドラッグして並べ替え、表示/非表示を切り替えられます。</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2246,6 +3116,16 @@
           <t>ユーザー名を変更できますか？</t>
         </is>
       </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>To change username: Settings &gt; Account &gt; Edit Profile &gt; Username. Note: you can only change it once every 30 days.</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>ユーザー名の変更：設定 &gt; アカウント &gt; プロフィール編集 &gt; ユーザー名。注意：変更は30日に1回のみ可能です。</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2268,6 +3148,16 @@
           <t>設定を開くと画面が真っ白になる</t>
         </is>
       </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>We're aware of display issues in settings. Try: 1) Clear app cache 2) Update to the latest version. Report at Settings &gt; Help &gt; Report a Bug with your device model.</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>設定画面の表示問題を認識しています。お試しください：1) アプリキャッシュを消去 2) 最新版にアップデート。デバイスモデルを添えて設定 &gt; ヘルプ &gt; バグを報告へ。</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2290,6 +3180,16 @@
           <t>ロード画面でフリーズする</t>
         </is>
       </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Loading screen freeze: try force closing and reopening the app. If it continues, clear the app cache or reinstall. Report at Settings &gt; Help &gt; Report a Bug.</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>ロード画面のフリーズ：アプリを強制終了して再起動してください。続く場合はキャッシュの消去または再インストールをお試しください。設定 &gt; ヘルプ &gt; バグを報告へ。</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2312,6 +3212,16 @@
           <t>エラーメッセージが出続けます</t>
         </is>
       </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Error messages can mean many things. Please note the exact error code/text and report it at Settings &gt; Help &gt; Report a Bug. We'll investigate ASAP.</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>エラーメッセージにはさまざまな原因があります。正確なエラーコード/テキストをメモして設定 &gt; ヘルプ &gt; バグを報告からご連絡ください。早急に調査します。</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2334,6 +3244,16 @@
           <t>ログインするたびにアプリが落ちる</t>
         </is>
       </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Login crashes: 1) Clear app cache 2) Check for updates 3) Try uninstalling and reinstalling. If it persists, report with device model at Settings &gt; Help &gt; Report a Bug.</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>ログイン時のクラッシュ：1) キャッシュ消去 2) アップデートを確認 3) アプリの再インストール。改善しない場合はデバイスモデルを添えて設定 &gt; ヘルプ &gt; バグを報告へ。</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2356,6 +3276,16 @@
           <t>ボタンが反応しない</t>
         </is>
       </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Unresponsive buttons: try scrolling to refresh the page, or force close and reopen the app. Report at Settings &gt; Help &gt; Report a Bug with your OS version.</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>ボタンが反応しない場合：ページをスクロールして更新するか、アプリを強制終了して再起動してください。OSバージョンを添えて設定 &gt; ヘルプ &gt; バグを報告へ。</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2378,6 +3308,16 @@
           <t>ページが正しく表示されない</t>
         </is>
       </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Page loading issues: check your internet connection first. Then try: 1) Clear app cache 2) Update the app. Report at Settings &gt; Help &gt; Report a Bug if it continues.</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>ページの読み込み問題：まずインターネット接続を確認。次に：1) キャッシュ消去 2) アプリ更新。続く場合は設定 &gt; ヘルプ &gt; バグを報告からご連絡ください。</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2400,6 +3340,16 @@
           <t>アップデート後にデータが消えた</t>
         </is>
       </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>We're sorry about the data loss! Please report immediately at Settings &gt; Help &gt; Report a Bug. Our team may be able to recover your data. Say 'I need human help' for urgent assistance.</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>データの消失について大変申し訳ございません！すぐに設定 &gt; ヘルプ &gt; バグを報告からご連絡ください。データの復旧が可能な場合があります。緊急の場合は「人と話したい」とお伝えください。</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2422,6 +3372,16 @@
           <t>表示にバグがあります</t>
         </is>
       </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Display glitches: try 1) Rotating your screen 2) Restarting the app 3) Updating to the latest version. Report with a screenshot at Settings &gt; Help &gt; Report a Bug.</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>表示の不具合：お試しください 1) 画面を回転 2) アプリを再起動 3) 最新版にアップデート。スクリーンショットを添えて設定 &gt; ヘルプ &gt; バグを報告へ。</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2444,6 +3404,16 @@
           <t>通知が届かなくなった</t>
         </is>
       </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Notification issues: check Settings &gt; Notifications are enabled, and verify your device allows notifications for our app. Try toggling off and on.</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>通知の問題：設定 &gt; 通知が有効になっているか確認し、デバイスのアプリ通知許可も確認してください。オフにしてからオンに切り替えてみてください。</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2466,6 +3436,16 @@
           <t>検索結果がおかしい</t>
         </is>
       </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Wrong search results: this may be a cache issue. Try clearing app cache at Settings &gt; General &gt; Clear Cache. If it persists, report at Settings &gt; Help &gt; Report a Bug.</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>検索結果の誤り：キャッシュの問題の可能性があります。設定 &gt; 一般 &gt; キャッシュ消去をお試しください。改善しない場合は設定 &gt; ヘルプ &gt; バグを報告へ。</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2488,6 +3468,16 @@
           <t>アプリで動画が再生されない</t>
         </is>
       </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Video playback issues: 1) Check internet connection 2) Try switching between Wi-Fi and mobile data 3) Clear app cache. Report at Settings &gt; Help &gt; Report a Bug.</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>動画再生の問題：1) インターネット接続を確認 2) Wi-Fiとモバイルデータを切り替え 3) キャッシュ消去。設定 &gt; ヘルプ &gt; バグを報告からご連絡ください。</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2510,6 +3500,16 @@
           <t>保存しようとするとエラーが出る</t>
         </is>
       </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Save errors: try 1) Check you have enough storage 2) Force close and retry 3) Check for app updates. Report at Settings &gt; Help &gt; Report a Bug with the error details.</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>保存エラー：お試しください 1) ストレージの空き容量を確認 2) 強制終了して再試行 3) アプリの更新を確認。エラー詳細を添えて設定 &gt; ヘルプ &gt; バグを報告へ。</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2532,6 +3532,16 @@
           <t>マネージャーと話させてください</t>
         </is>
       </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>I understand your frustration. I'll escalate this to a senior team member. Please submit details at Settings &gt; Help &gt; Contact Support and mark it as urgent.</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>ご不満をお察しします。上級チームメンバーにエスカレートいたします。設定 &gt; ヘルプ &gt; サポートに連絡から詳細を送信し、緊急としてマークしてください。</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2554,6 +3564,16 @@
           <t>苦情を申し立てたい</t>
         </is>
       </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>I'm sorry you're having trouble. To file a complaint: Settings &gt; Help &gt; Contact Support &gt; select 'Complaint'. We take all feedback seriously.</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>ご迷惑をおかけして申し訳ございません。苦情を提出するには：設定 &gt; ヘルプ &gt; サポートに連絡 &gt; 「苦情」を選択。すべてのフィードバックを真摯に受け止めています。</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2576,6 +3596,16 @@
           <t>このボットでは解決できません</t>
         </is>
       </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>I understand! Let me connect you with our team. Please reach out at Settings &gt; Help &gt; Contact Support for personalized help within 24 hours.</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>かしこまりました！チームにおつなぎします。設定 &gt; ヘルプ &gt; サポートに連絡から、24時間以内に個別対応いたします。</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2598,6 +3628,16 @@
           <t>人間のオペレーターに転送して</t>
         </is>
       </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Transferring you! Please contact our team at Settings &gt; Help &gt; Contact Support. Include your account email for faster service.</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>おつなぎします！設定 &gt; ヘルプ &gt; サポートに連絡からチームにご連絡ください。アカウントメールを記載いただくと迅速に対応できます。</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2620,6 +3660,16 @@
           <t>本物の人と話す必要があります</t>
         </is>
       </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Of course! Our team is available at Settings &gt; Help &gt; Contact Support. Response time is within 24 hours, urgent issues are prioritized.</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>もちろんです！設定 &gt; ヘルプ &gt; サポートに連絡からチームにご連絡いただけます。24時間以内に対応し、緊急の問題は優先されます。</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2642,6 +3692,16 @@
           <t>カスタマーサービスに電話できますか？</t>
         </is>
       </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Phone support is available Mon-Fri 9AM-6PM (JST). You can also reach us via Settings &gt; Help &gt; Contact Support for 24/7 chat assistance.</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>電話サポートは月〜金 9:00-18:00（JST）で対応しています。設定 &gt; ヘルプ &gt; サポートに連絡から24時間チャットもご利用いただけます。</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2664,6 +3724,16 @@
           <t>折り返し電話がほしい</t>
         </is>
       </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>We can arrange a callback! Please submit your request at Settings &gt; Help &gt; Contact Support &gt; select 'Request Callback'. Include your phone number and preferred time.</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>コールバックを手配できます！設定 &gt; ヘルプ &gt; サポートに連絡 &gt; 「コールバックリクエスト」を選択。電話番号とご希望の時間をお知らせください。</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -2686,6 +3756,16 @@
           <t>問題をエスカレートしてください</t>
         </is>
       </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>I'll escalate your issue right away. Please provide details at Settings &gt; Help &gt; Contact Support and mark the priority as 'High'.</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>すぐに問題をエスカレートします。設定 &gt; ヘルプ &gt; サポートに連絡で詳細をお知らせいただき、優先度を「高」に設定してください。</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -2708,6 +3788,16 @@
           <t>ライブチャットはありますか？</t>
         </is>
       </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Yes! Live chat is available at Settings &gt; Help &gt; Live Chat during business hours (Mon-Fri 9AM-6PM JST). Outside hours, use Contact Support for async help.</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>はい！ライブチャットは営業時間中（月〜金 9:00-18:00 JST）に設定 &gt; ヘルプ &gt; ライブチャットからご利用いただけます。営業時間外はサポートに連絡をご利用ください。</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2730,6 +3820,16 @@
           <t>ボットでは対応できない問題です</t>
         </is>
       </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>I understand — some issues need a personal touch. Please describe your situation at Settings &gt; Help &gt; Contact Support. Our experts will handle it.</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>かしこまりました。個別対応が必要な問題もございます。設定 &gt; ヘルプ &gt; サポートに連絡で状況をお知らせください。専門スタッフが対応いたします。</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2752,6 +3852,16 @@
           <t>実際のスタッフにつないでください</t>
         </is>
       </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Connecting you with a real agent! Please submit your request at Settings &gt; Help &gt; Contact Support. Include your issue summary for faster help.</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>実際のエージェントにおつなぎします！設定 &gt; ヘルプ &gt; サポートに連絡からリクエストを送信してください。問題の概要を記載いただくと迅速に対応できます。</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2774,6 +3884,16 @@
           <t>個別のサポートが必要です</t>
         </is>
       </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Of course! For personalized assistance, reach our team at Settings &gt; Help &gt; Contact Support. They'll work with you one-on-one to resolve your issue.</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>もちろんです！個別対応は設定 &gt; ヘルプ &gt; サポートに連絡からチームにご連絡ください。マンツーマンで問題解決にあたります。</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -2796,6 +3916,16 @@
           <t>フランスの首都はどこ？</t>
         </is>
       </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Geography isn't my specialty — app support is! Ask me about accounts, subscriptions, billing, features, or bugs.</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>地理は専門外ですが、アプリサポートなら任せてください！アカウント、サブスクリプション、請求、機能、バグについてお聞きください。</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -2818,6 +3948,16 @@
           <t>音楽を再生して</t>
         </is>
       </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>I can't play music, but I can help with your app experience! What do you need help with?</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>音楽は再生できませんが、アプリのご利用についてお手伝いできます！何かお困りですか？</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2840,6 +3980,16 @@
           <t>今日の株式市場はどう？</t>
         </is>
       </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Stock market isn't my area — I'm here for app support! Ask about accounts, billing, features, or report issues.</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>株式市場は専門外です。アプリサポートならお任せください！アカウント、請求、機能、問題報告についてお聞きください。</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -2862,6 +4012,16 @@
           <t>エッセイを書いて</t>
         </is>
       </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Essay writing is beyond my abilities! But I'm great at helping with your app. What can I assist you with?</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>エッセイの作成はできませんが、アプリのお手伝いなら得意です！何かお手伝いできることはありますか？</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -2884,6 +4044,16 @@
           <t>これをスペイン語に翻訳して</t>
         </is>
       </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>I can't translate, but I can help in both English and Japanese for app support! What do you need?</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>翻訳はできませんが、アプリサポートは英語と日本語の両方で対応できます！何かお困りですか？</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -2906,6 +4076,16 @@
           <t>飛行機を予約して</t>
         </is>
       </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>I can't book flights, but I can help with your app account, subscription, billing, or features!</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>航空券の予約はできませんが、アプリのアカウント、サブスクリプション、請求、機能についてお手伝いできます！</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -2928,6 +4108,16 @@
           <t>2+2は？</t>
         </is>
       </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Math isn't my thing — app support is! Ask me about passwords, subscriptions, billing, or app features.</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>計算は専門外です。アプリサポートならお任せください！パスワード、サブスクリプション、請求、機能についてお聞きください。</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -2950,6 +4140,16 @@
           <t>午前7時にアラームをセットして</t>
         </is>
       </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>I can't set alarms, but I can help you get the most out of your app! What would you like to know?</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>アラームは設定できませんが、アプリの活用方法ならお手伝いできます！何をお知りになりたいですか？</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -2972,6 +4172,16 @@
           <t>大統領は誰？</t>
         </is>
       </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>I don't follow politics, but I'm an expert at app support! Ask about accounts, billing, features, or bugs.</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>政治には詳しくないですが、アプリサポートなら専門家です！アカウント、請求、機能、バグについてお聞きください。</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -2992,6 +4202,16 @@
       <c r="D132" t="inlineStr">
         <is>
           <t>近くのレストランを探して</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>I can't find restaurants, but I can navigate your app! Ask about settings, features, account, or billing.</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>レストラン検索はできませんが、アプリのナビゲートならお任せください！設定、機能、アカウント、請求についてお聞きください。</t>
         </is>
       </c>
     </row>

</xml_diff>